<commit_message>
Añadiendo campos nuevos a la compañía y a las vistas e importador
</commit_message>
<xml_diff>
--- a/krm/static/files/import_companies.xlsx
+++ b/krm/static/files/import_companies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bienvenidosaez/Bitbucket/krm-kpmg/krm/static/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E749C0A0-8B81-1246-A11D-1B1C102A6DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6287C95-0338-9F4C-BB3F-1CB76C727AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25100" yWindow="4400" windowWidth="46600" windowHeight="22800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compañías" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="511">
   <si>
     <t>VAT</t>
   </si>
@@ -1583,6 +1583,12 @@
   </si>
   <si>
     <t>REF</t>
+  </si>
+  <si>
+    <t>TIPO</t>
+  </si>
+  <si>
+    <t>COMPANIES IN SCOPE</t>
   </si>
 </sst>
 </file>
@@ -2088,7 +2094,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:K1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" style="2" customWidth="1"/>
@@ -2100,9 +2106,10 @@
     <col min="7" max="7" width="9" style="9" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="31" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="26.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="32.5" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1"/>
       <c r="B1" s="11" t="s">
         <v>2</v>
@@ -2114,8 +2121,10 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
       <c r="I1" s="12"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1"/>
+      <c r="K1"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>508</v>
       </c>
@@ -2143,85 +2152,91 @@
       <c r="I2" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="E3" s="3"/>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G4" s="9" t="str">
-        <f t="shared" ref="G3:G66" si="0">IF(ISBLANK(H4),"",VLOOKUP(H4,PAISES,2))</f>
+        <f t="shared" ref="G4:G66" si="0">IF(ISBLANK(H4),"",VLOOKUP(H4,PAISES,2))</f>
         <v/>
       </c>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G5" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G6" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G7" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G8" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G9" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G10" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G11" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G12" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G13" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G14" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G15" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G16" s="9" t="str">
         <f t="shared" si="0"/>
         <v/>

</xml_diff>